<commit_message>
hkr apc data 2025 processed, changed yes no is_hybrid in original data
</commit_message>
<xml_diff>
--- a/data/hkr/original_data/HKR_OpenAPC_2025.xlsx
+++ b/data/hkr/original_data/HKR_OpenAPC_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\hkr.se\home$\pah\Documents\OpenAPC HKR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/2021m30/R/repos/openapc-se/data/hkr/original_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63722FE-83AC-43E9-A130-C22990BFE4A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1663761E-738A-7A4D-B03B-0762A058E816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="80920" yWindow="2920" windowWidth="23260" windowHeight="13900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="article data" sheetId="1" r:id="rId1"/>
@@ -122,9 +122,6 @@
     <t>10.1080/2331186X.2025.2457290</t>
   </si>
   <si>
-    <t>no</t>
-  </si>
-  <si>
     <t>Taylor &amp; Francis</t>
   </si>
   <si>
@@ -140,9 +137,6 @@
     <t>10.1080/13504622.2025.2505188</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Environmental Education Research</t>
   </si>
   <si>
@@ -171,6 +165,12 @@
   </si>
   <si>
     <t>IJREE – International Journal for Research on Extended Education</t>
+  </si>
+  <si>
+    <t>False</t>
+  </si>
+  <si>
+    <t>True</t>
   </si>
 </sst>
 </file>
@@ -256,17 +256,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -559,22 +557,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="10.59765625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.09765625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.796875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="26.8984375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.83203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="26.83203125" style="2" customWidth="1"/>
     <col min="5" max="6" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5" style="8" customWidth="1"/>
-    <col min="8" max="8" width="5.09765625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.59765625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.8984375" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.3984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5" style="2" customWidth="1"/>
+    <col min="8" max="8" width="5.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="11" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" ht="15.6">
+    <row r="1" spans="1:11" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -593,7 +591,7 @@
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -609,7 +607,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="30">
+    <row r="2" spans="1:11" ht="34">
       <c r="A2" s="2" t="s">
         <v>20</v>
       </c>
@@ -619,29 +617,29 @@
       <c r="C2" s="4">
         <v>3375</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="9" t="s">
         <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="H2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="J2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="J2" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>26</v>
-      </c>
     </row>
-    <row r="3" spans="1:11" ht="15.6">
+    <row r="3" spans="1:11">
       <c r="A3" s="2" t="s">
         <v>20</v>
       </c>
@@ -652,31 +650,31 @@
         <v>24817</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="H3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="9" t="s">
+      <c r="I3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="K3" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>32</v>
-      </c>
     </row>
-    <row r="4" spans="1:11" ht="15.6">
+    <row r="4" spans="1:11">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -687,28 +685,28 @@
         <v>7342</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="H4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="I4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="K4" s="6" t="s">
         <v>36</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -724,18 +722,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E9D608-332C-6B41-B918-E0AD75CD6855}">
   <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultColWidth="10.8984375" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="4" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.8984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.8984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.59765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="7.8984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="10.8984375" style="1"/>
+    <col min="9" max="10" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">

</xml_diff>